<commit_message>
Replace the made-up demo contacts with real Nile wallets named Dummy 1 to 6
setup --force-data now creates the demo contacts as real keypairs and saves
their private keys in backend/data/demo-wallets.local.json (git-ignored), so
a demo wallet can be opened in TronLink. The address-poisoning row still
works: a birthday search over consecutive keys finds a real wallet pair that
shares its first and last four characters, in about two minutes.

Also: signing payment limits returns at once and the registry record lands
in the background; confirmations read the full node, which answers within a
block instead of after the one-minute solidification.
</commit_message>
<xml_diff>
--- a/backend/data/demo/ansim-demo-payouts.xlsx
+++ b/backend/data/demo/ansim-demo-payouts.xlsx
@@ -418,13 +418,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Nguyen Van An</v>
+        <v>Sender 1</v>
       </c>
       <c r="B2" t="str">
-        <v>Nguyen Thi Lan</v>
+        <v>Dummy 1</v>
       </c>
       <c r="C2" t="str">
-        <v>TXZit1DZuH3oLxZmxooogX3Uh5nuYiXDVt</v>
+        <v>TWTRqGYVDY6MHkcRH8iRBJcX3kWbNFp6Pz</v>
       </c>
       <c r="D2" t="str">
         <v>3.00</v>
@@ -435,13 +435,13 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Tran Quoc Bao</v>
+        <v>Sender 2</v>
       </c>
       <c r="B3" t="str">
-        <v>Tran Van Minh</v>
+        <v>Dummy 2</v>
       </c>
       <c r="C3" t="str">
-        <v>TUQjGCvRobwtagKYNJVncoG9VkwdM6csZN</v>
+        <v>TC12C8b3ucM7LwDQnPQDKDR8qSjUunz2P1</v>
       </c>
       <c r="D3" t="str">
         <v>2.50</v>
@@ -452,13 +452,13 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Maria Reyes</v>
+        <v>Sender 3</v>
       </c>
       <c r="B4" t="str">
-        <v>Maria Santos</v>
+        <v>Dummy 3</v>
       </c>
       <c r="C4" t="str">
-        <v>TMNLjjbCGAtFi9dnPPbsxVoXZCx3ZUcSYD</v>
+        <v>TQYJVPVr89y8qwSvQi4denhy7hV1GKQGVe</v>
       </c>
       <c r="D4" t="str">
         <v>2.00</v>
@@ -469,13 +469,13 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Bikash Gurung</v>
+        <v>Sender 4</v>
       </c>
       <c r="B5" t="str">
-        <v>Sita Gurung</v>
+        <v>Dummy 4</v>
       </c>
       <c r="C5" t="str">
-        <v>TT2oDJK26u2W1F9uLbHq1xpMacWrefSjy4</v>
+        <v>TMHtqxZS7swQ79aqwyFDsRad7VgpfLBuoa</v>
       </c>
       <c r="D5" t="str">
         <v>10.00</v>
@@ -486,13 +486,13 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Tran Quoc Bao</v>
+        <v>Sender 2</v>
       </c>
       <c r="B6" t="str">
-        <v>Tran Van Minh</v>
+        <v>Dummy 2</v>
       </c>
       <c r="C6" t="str">
-        <v>TUQjGCvRobwtagKYNJVncoG9VkwdM6csZN</v>
+        <v>TC12C8b3ucM7LwDQnPQDKDR8qSjUunz2P1</v>
       </c>
       <c r="D6" t="str">
         <v>2.50</v>
@@ -503,13 +503,13 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Nguyen Van An</v>
+        <v>Sender 1</v>
       </c>
       <c r="B7" t="str">
-        <v>Nguyen Thi Lan</v>
+        <v>Dummy 1</v>
       </c>
       <c r="C7" t="str">
-        <v>TXZiWc1wHoxz5dj8WeZZyhUBLE3VV8XDVt</v>
+        <v>TWTRG6z4ybC7nFNrDR6TRkk8UEgzHpp6Pz</v>
       </c>
       <c r="D7" t="str">
         <v>3.00</v>
@@ -520,13 +520,13 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Juan Cruz</v>
+        <v>Sender 5</v>
       </c>
       <c r="B8" t="str">
-        <v>Juan dela Cruz</v>
+        <v>Dummy 5</v>
       </c>
       <c r="C8" t="str">
-        <v>TE1Vq6e6JwZGd55J2N1Cux7D1SV5mMQdQH</v>
+        <v>TWRMWKCUWnrvWeoFmFC2rGhEgFRWgqviem</v>
       </c>
       <c r="D8" t="str">
         <v>2.00</v>
@@ -537,13 +537,13 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>김민수</v>
+        <v>Sender 7</v>
       </c>
       <c r="B9" t="str">
-        <v>Le Van Hung</v>
+        <v>Dummy 7</v>
       </c>
       <c r="C9" t="str">
-        <v>TGAioN85pbuLoiBZiF36oDYtr4Li75Y5MM</v>
+        <v>TMamw7bcB8Fd9g1fAh5R97RoXPyPDLXs2K</v>
       </c>
       <c r="D9" t="str">
         <v>1.00</v>
@@ -554,13 +554,13 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>박지훈</v>
+        <v>Sender 8</v>
       </c>
       <c r="B10" t="str">
-        <v>Le Van Hung</v>
+        <v>Dummy 7</v>
       </c>
       <c r="C10" t="str">
-        <v>TGAioN85pbuLoiBZiF36oDYtr4Li75Y5MM</v>
+        <v>TMamw7bcB8Fd9g1fAh5R97RoXPyPDLXs2K</v>
       </c>
       <c r="D10" t="str">
         <v>1.00</v>
@@ -571,13 +571,13 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>최서연</v>
+        <v>Sender 9</v>
       </c>
       <c r="B11" t="str">
-        <v>Le Van Hung</v>
+        <v>Dummy 7</v>
       </c>
       <c r="C11" t="str">
-        <v>TGAioN85pbuLoiBZiF36oDYtr4Li75Y5MM</v>
+        <v>TMamw7bcB8Fd9g1fAh5R97RoXPyPDLXs2K</v>
       </c>
       <c r="D11" t="str">
         <v>1.00</v>
@@ -588,13 +588,13 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Sokha Chan</v>
+        <v>Sender 10</v>
       </c>
       <c r="B12" t="str">
-        <v>Chan Dara</v>
+        <v>Dummy 8</v>
       </c>
       <c r="C12" t="str">
-        <v>TPJjH3zykTkZ9NsgPo115kU5PxCfuyTjEd</v>
+        <v>TSSJ4FADxu3dToKDtBivTpWkqNYieDofem</v>
       </c>
       <c r="D12" t="str">
         <v>2.00</v>
@@ -605,13 +605,13 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Aung Min</v>
+        <v>Sender 11</v>
       </c>
       <c r="B13" t="str">
-        <v>Hla Hla</v>
+        <v>Dummy 9</v>
       </c>
       <c r="C13" t="str">
-        <v>TQV2zHvMsK3GAm1LYkhNPnec1mxjpvJsgt</v>
+        <v>TSPXmqBRyn8D8Tb6HRVxMbrsCqiUVHFU5i</v>
       </c>
       <c r="D13" t="str">
         <v>1.50</v>
@@ -622,13 +622,13 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Ram Bahadur</v>
+        <v>Sender 6</v>
       </c>
       <c r="B14" t="str">
-        <v>Ram Thapa</v>
+        <v>Dummy 6</v>
       </c>
       <c r="C14" t="str">
-        <v>TL2h4YmbDnANRJ7xqYqUiTtmqFF78argyw</v>
+        <v>TYTGczFG86EWhBaBkMtrXhATVf6pfkJT6m</v>
       </c>
       <c r="D14" t="str">
         <v>2.00</v>

</xml_diff>